<commit_message>
feat: configure question count per difficulty, support images in study steps, and update excel import
</commit_message>
<xml_diff>
--- a/public/ProEdu_Import_Procvicovani.xlsx
+++ b/public/ProEdu_Import_Procvicovani.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -439,6 +439,9 @@
       <c r="M1" t="str">
         <v>Odpověď (výběr)</v>
       </c>
+      <c r="N1" t="str">
+        <v>Obtížnost</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -480,6 +483,9 @@
       <c r="M2" t="str">
         <v>B</v>
       </c>
+      <c r="N2" t="str">
+        <v>Lehká</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -521,6 +527,9 @@
       <c r="M3" t="str">
         <v/>
       </c>
+      <c r="N3" t="str">
+        <v>Střední</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -562,10 +571,13 @@
       <c r="M4" t="str">
         <v>B</v>
       </c>
+      <c r="N4" t="str">
+        <v>Lehká</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>